<commit_message>
Congelar regressao 7 ativos e fixtures
</commit_message>
<xml_diff>
--- a/tests/fixtures/posicao_7_ativos.xlsx
+++ b/tests/fixtures/posicao_7_ativos.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Acoes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="BDR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tesouro Direto" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -502,7 +503,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>5589656</t>
+          <t>0000000</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -566,7 +567,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>5589656</t>
+          <t>0000000</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -630,7 +631,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5589656</t>
+          <t>0000000</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -694,7 +695,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5589656</t>
+          <t>0000000</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -839,7 +840,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>5589656</t>
+          <t>0000000</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -898,7 +899,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>5589656</t>
+          <t>0000000</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -957,7 +958,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5589656</t>
+          <t>0000000</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1001,6 +1002,87 @@
       </c>
       <c r="M4" t="n">
         <v>251</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Instituição</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Código ISIN</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Indexador</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Vencimento</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Quantidade</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Quantidade Disponível</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Quantidade Indisponível</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Motivo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Valor Aplicado</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Valor bruto</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Valor líquido</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Valor Atualizado</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>